<commit_message>
Update Italy report data pipeline outputs
</commit_message>
<xml_diff>
--- a/OECD-Reports/main_indicators.xlsx
+++ b/OECD-Reports/main_indicators.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10525"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wjproject.sharepoint.com/research/Programmatic/Data Analytics/6. Country Reports/OECD-EULNS/output/tabs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wjproject.sharepoint.com/research/Programmatic/Data Analytics/6. Country Reports/OECD-EULNS/OECD-Reports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_874FC65F1A70086B2B689FC427983F5EB0277B3D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59D08F24-2CAB-D448-AB43-89AEBCF4001D}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="11_874FC65F1A70086B2B689FC427983F5EB0277B3D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{62916463-193C-F944-A0D9-FB2804CEA364}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28800" yWindow="-3600" windowWidth="38400" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="visual_indicators" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">visual_indicators!$D$1:$D$569</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">visual_indicators!$A$1:$H$569</definedName>
   </definedNames>
   <calcPr calcId="124519"/>
 </workbook>
@@ -876,7 +876,7 @@
         <v>12</v>
       </c>
       <c r="G2">
-        <v>58.080942553070066</v>
+        <v>58.080942553070102</v>
       </c>
       <c r="H2">
         <v>3820</v>
@@ -934,7 +934,7 @@
         <v>5252</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -960,7 +960,7 @@
         <v>3844</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -986,7 +986,7 @@
         <v>3844</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1012,7 +1012,7 @@
         <v>3844</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1038,7 +1038,7 @@
         <v>3844</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -1064,7 +1064,7 @@
         <v>3844</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1090,7 +1090,7 @@
         <v>3844</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -1116,7 +1116,7 @@
         <v>3844</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -1142,7 +1142,7 @@
         <v>3844</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -1168,7 +1168,7 @@
         <v>3844</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -1194,7 +1194,7 @@
         <v>3844</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -1220,7 +1220,7 @@
         <v>3844</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -1870,7 +1870,7 @@
         <v>5252</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>30</v>
       </c>
@@ -1896,7 +1896,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>30</v>
       </c>
@@ -1922,7 +1922,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>30</v>
       </c>
@@ -1948,7 +1948,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>30</v>
       </c>
@@ -1974,7 +1974,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>30</v>
       </c>
@@ -1997,7 +1997,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>30</v>
       </c>
@@ -2023,7 +2023,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>30</v>
       </c>
@@ -2049,7 +2049,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>30</v>
       </c>
@@ -2075,7 +2075,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>30</v>
       </c>
@@ -2101,7 +2101,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>30</v>
       </c>
@@ -2124,7 +2124,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>30</v>
       </c>
@@ -2150,7 +2150,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>30</v>
       </c>
@@ -2902,7 +2902,7 @@
         <v>2644</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>36</v>
       </c>
@@ -2925,7 +2925,7 @@
         <v>1637</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>36</v>
       </c>
@@ -2948,7 +2948,7 @@
         <v>1637</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>36</v>
       </c>
@@ -2971,7 +2971,7 @@
         <v>1637</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>36</v>
       </c>
@@ -2997,7 +2997,7 @@
         <v>1637</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>36</v>
       </c>
@@ -3020,7 +3020,7 @@
         <v>1637</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>36</v>
       </c>
@@ -3046,7 +3046,7 @@
         <v>1637</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>36</v>
       </c>
@@ -3072,7 +3072,7 @@
         <v>1637</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>36</v>
       </c>
@@ -3095,7 +3095,7 @@
         <v>1637</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>36</v>
       </c>
@@ -3121,7 +3121,7 @@
         <v>1637</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>36</v>
       </c>
@@ -3144,7 +3144,7 @@
         <v>1637</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>36</v>
       </c>
@@ -3170,7 +3170,7 @@
         <v>1637</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>36</v>
       </c>
@@ -3838,7 +3838,7 @@
         <v>862</v>
       </c>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>36</v>
       </c>
@@ -3864,7 +3864,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>36</v>
       </c>
@@ -3890,7 +3890,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>36</v>
       </c>
@@ -3916,7 +3916,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>36</v>
       </c>
@@ -3942,7 +3942,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>36</v>
       </c>
@@ -3968,7 +3968,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>36</v>
       </c>
@@ -3994,7 +3994,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>36</v>
       </c>
@@ -4020,7 +4020,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="129" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>36</v>
       </c>
@@ -5190,7 +5190,7 @@
         <v>1505</v>
       </c>
     </row>
-    <row r="174" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>64</v>
       </c>
@@ -5213,7 +5213,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="175" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>64</v>
       </c>
@@ -5236,7 +5236,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="176" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>64</v>
       </c>
@@ -5259,7 +5259,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="177" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>64</v>
       </c>
@@ -5282,7 +5282,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="178" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>64</v>
       </c>
@@ -5305,7 +5305,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="179" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>64</v>
       </c>
@@ -5328,7 +5328,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="180" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>64</v>
       </c>
@@ -5354,7 +5354,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="181" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>64</v>
       </c>
@@ -5377,7 +5377,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="182" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>64</v>
       </c>
@@ -5400,7 +5400,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="183" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>64</v>
       </c>
@@ -5423,7 +5423,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="184" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>64</v>
       </c>
@@ -5449,7 +5449,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="185" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
         <v>64</v>
       </c>
@@ -6105,7 +6105,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="213" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
         <v>64</v>
       </c>
@@ -6131,7 +6131,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="214" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
         <v>64</v>
       </c>
@@ -6157,7 +6157,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="215" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
         <v>64</v>
       </c>
@@ -6183,7 +6183,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="216" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
         <v>64</v>
       </c>
@@ -6209,7 +6209,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="217" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
         <v>64</v>
       </c>
@@ -6495,7 +6495,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="228" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
         <v>64</v>
       </c>
@@ -6521,7 +6521,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="229" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
         <v>64</v>
       </c>
@@ -6547,7 +6547,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="230" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
         <v>64</v>
       </c>
@@ -6573,7 +6573,7 @@
         <v>2071</v>
       </c>
     </row>
-    <row r="231" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
         <v>64</v>
       </c>
@@ -6599,7 +6599,7 @@
         <v>2071</v>
       </c>
     </row>
-    <row r="232" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
         <v>64</v>
       </c>
@@ -6625,7 +6625,7 @@
         <v>2071</v>
       </c>
     </row>
-    <row r="233" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
         <v>64</v>
       </c>
@@ -6651,7 +6651,7 @@
         <v>2071</v>
       </c>
     </row>
-    <row r="234" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
         <v>64</v>
       </c>
@@ -7041,7 +7041,7 @@
         <v>1475</v>
       </c>
     </row>
-    <row r="249" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
         <v>84</v>
       </c>
@@ -7064,7 +7064,7 @@
         <v>1271</v>
       </c>
     </row>
-    <row r="250" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
         <v>84</v>
       </c>
@@ -7087,7 +7087,7 @@
         <v>1271</v>
       </c>
     </row>
-    <row r="251" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
         <v>84</v>
       </c>
@@ -7110,7 +7110,7 @@
         <v>1271</v>
       </c>
     </row>
-    <row r="252" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
         <v>84</v>
       </c>
@@ -7136,7 +7136,7 @@
         <v>1271</v>
       </c>
     </row>
-    <row r="253" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
         <v>84</v>
       </c>
@@ -7159,7 +7159,7 @@
         <v>1271</v>
       </c>
     </row>
-    <row r="254" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A254" t="s">
         <v>84</v>
       </c>
@@ -7182,7 +7182,7 @@
         <v>1271</v>
       </c>
     </row>
-    <row r="255" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
         <v>84</v>
       </c>
@@ -7208,7 +7208,7 @@
         <v>1271</v>
       </c>
     </row>
-    <row r="256" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A256" t="s">
         <v>84</v>
       </c>
@@ -7231,7 +7231,7 @@
         <v>1271</v>
       </c>
     </row>
-    <row r="257" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A257" t="s">
         <v>84</v>
       </c>
@@ -7254,7 +7254,7 @@
         <v>1271</v>
       </c>
     </row>
-    <row r="258" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A258" t="s">
         <v>84</v>
       </c>
@@ -7277,7 +7277,7 @@
         <v>1271</v>
       </c>
     </row>
-    <row r="259" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A259" t="s">
         <v>84</v>
       </c>
@@ -7303,7 +7303,7 @@
         <v>1271</v>
       </c>
     </row>
-    <row r="260" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A260" t="s">
         <v>84</v>
       </c>
@@ -7971,7 +7971,7 @@
         <v>1045</v>
       </c>
     </row>
-    <row r="288" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A288" t="s">
         <v>84</v>
       </c>
@@ -7994,7 +7994,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="289" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A289" t="s">
         <v>84</v>
       </c>
@@ -8017,7 +8017,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="290" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A290" t="s">
         <v>84</v>
       </c>
@@ -8040,7 +8040,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="291" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A291" t="s">
         <v>84</v>
       </c>
@@ -8066,7 +8066,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="292" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A292" t="s">
         <v>84</v>
       </c>
@@ -8089,7 +8089,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="293" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A293" t="s">
         <v>84</v>
       </c>
@@ -8112,7 +8112,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="294" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A294" t="s">
         <v>84</v>
       </c>
@@ -8138,7 +8138,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="295" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A295" t="s">
         <v>84</v>
       </c>
@@ -8161,7 +8161,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="296" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A296" t="s">
         <v>84</v>
       </c>
@@ -8184,7 +8184,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="297" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A297" t="s">
         <v>84</v>
       </c>
@@ -8207,7 +8207,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="298" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A298" t="s">
         <v>84</v>
       </c>
@@ -8233,7 +8233,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="299" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A299" t="s">
         <v>84</v>
       </c>
@@ -8901,7 +8901,7 @@
         <v>1050</v>
       </c>
     </row>
-    <row r="327" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="327" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A327" t="s">
         <v>84</v>
       </c>
@@ -8924,7 +8924,7 @@
         <v>1336</v>
       </c>
     </row>
-    <row r="328" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="328" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A328" t="s">
         <v>84</v>
       </c>
@@ -8947,7 +8947,7 @@
         <v>1336</v>
       </c>
     </row>
-    <row r="329" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="329" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A329" t="s">
         <v>84</v>
       </c>
@@ -8970,7 +8970,7 @@
         <v>1336</v>
       </c>
     </row>
-    <row r="330" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="330" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A330" t="s">
         <v>84</v>
       </c>
@@ -8996,7 +8996,7 @@
         <v>1336</v>
       </c>
     </row>
-    <row r="331" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="331" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A331" t="s">
         <v>84</v>
       </c>
@@ -9019,7 +9019,7 @@
         <v>1336</v>
       </c>
     </row>
-    <row r="332" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="332" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A332" t="s">
         <v>84</v>
       </c>
@@ -9042,7 +9042,7 @@
         <v>1336</v>
       </c>
     </row>
-    <row r="333" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="333" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A333" t="s">
         <v>84</v>
       </c>
@@ -9068,7 +9068,7 @@
         <v>1336</v>
       </c>
     </row>
-    <row r="334" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="334" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A334" t="s">
         <v>84</v>
       </c>
@@ -9091,7 +9091,7 @@
         <v>1336</v>
       </c>
     </row>
-    <row r="335" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="335" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A335" t="s">
         <v>84</v>
       </c>
@@ -9114,7 +9114,7 @@
         <v>1336</v>
       </c>
     </row>
-    <row r="336" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="336" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A336" t="s">
         <v>84</v>
       </c>
@@ -9137,7 +9137,7 @@
         <v>1336</v>
       </c>
     </row>
-    <row r="337" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="337" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A337" t="s">
         <v>84</v>
       </c>
@@ -9163,7 +9163,7 @@
         <v>1336</v>
       </c>
     </row>
-    <row r="338" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="338" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A338" t="s">
         <v>84</v>
       </c>
@@ -9831,7 +9831,7 @@
         <v>1059</v>
       </c>
     </row>
-    <row r="366" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="366" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A366" t="s">
         <v>84</v>
       </c>
@@ -9854,7 +9854,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="367" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="367" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A367" t="s">
         <v>84</v>
       </c>
@@ -9877,7 +9877,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="368" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="368" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A368" t="s">
         <v>84</v>
       </c>
@@ -9900,7 +9900,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="369" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="369" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A369" t="s">
         <v>84</v>
       </c>
@@ -9926,7 +9926,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="370" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="370" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A370" t="s">
         <v>84</v>
       </c>
@@ -9949,7 +9949,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="371" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="371" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A371" t="s">
         <v>84</v>
       </c>
@@ -9972,7 +9972,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="372" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="372" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A372" t="s">
         <v>84</v>
       </c>
@@ -9998,7 +9998,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="373" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="373" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A373" t="s">
         <v>84</v>
       </c>
@@ -10021,7 +10021,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="374" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="374" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A374" t="s">
         <v>84</v>
       </c>
@@ -10044,7 +10044,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="375" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="375" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A375" t="s">
         <v>84</v>
       </c>
@@ -10067,7 +10067,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="376" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="376" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A376" t="s">
         <v>84</v>
       </c>
@@ -10093,7 +10093,7 @@
         <v>1324</v>
       </c>
     </row>
-    <row r="377" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="377" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A377" t="s">
         <v>84</v>
       </c>
@@ -10761,7 +10761,7 @@
         <v>1045</v>
       </c>
     </row>
-    <row r="405" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="405" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A405" t="s">
         <v>84</v>
       </c>
@@ -10784,7 +10784,7 @@
         <v>1330</v>
       </c>
     </row>
-    <row r="406" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="406" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A406" t="s">
         <v>84</v>
       </c>
@@ -10807,7 +10807,7 @@
         <v>1330</v>
       </c>
     </row>
-    <row r="407" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="407" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A407" t="s">
         <v>84</v>
       </c>
@@ -10830,7 +10830,7 @@
         <v>1330</v>
       </c>
     </row>
-    <row r="408" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="408" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A408" t="s">
         <v>84</v>
       </c>
@@ -10856,7 +10856,7 @@
         <v>1330</v>
       </c>
     </row>
-    <row r="409" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="409" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A409" t="s">
         <v>84</v>
       </c>
@@ -10879,7 +10879,7 @@
         <v>1330</v>
       </c>
     </row>
-    <row r="410" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="410" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A410" t="s">
         <v>84</v>
       </c>
@@ -10902,7 +10902,7 @@
         <v>1330</v>
       </c>
     </row>
-    <row r="411" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="411" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A411" t="s">
         <v>84</v>
       </c>
@@ -10928,7 +10928,7 @@
         <v>1330</v>
       </c>
     </row>
-    <row r="412" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="412" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A412" t="s">
         <v>84</v>
       </c>
@@ -10951,7 +10951,7 @@
         <v>1330</v>
       </c>
     </row>
-    <row r="413" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="413" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A413" t="s">
         <v>84</v>
       </c>
@@ -10974,7 +10974,7 @@
         <v>1330</v>
       </c>
     </row>
-    <row r="414" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="414" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A414" t="s">
         <v>84</v>
       </c>
@@ -10997,7 +10997,7 @@
         <v>1330</v>
       </c>
     </row>
-    <row r="415" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="415" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A415" t="s">
         <v>84</v>
       </c>
@@ -11023,7 +11023,7 @@
         <v>1330</v>
       </c>
     </row>
-    <row r="416" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="416" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A416" t="s">
         <v>84</v>
       </c>
@@ -11691,7 +11691,7 @@
         <v>1056</v>
       </c>
     </row>
-    <row r="444" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="444" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A444" t="s">
         <v>95</v>
       </c>
@@ -11714,7 +11714,7 @@
         <v>1338</v>
       </c>
     </row>
-    <row r="445" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="445" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A445" t="s">
         <v>95</v>
       </c>
@@ -11737,7 +11737,7 @@
         <v>1338</v>
       </c>
     </row>
-    <row r="446" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="446" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A446" t="s">
         <v>95</v>
       </c>
@@ -11760,7 +11760,7 @@
         <v>1338</v>
       </c>
     </row>
-    <row r="447" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="447" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A447" t="s">
         <v>95</v>
       </c>
@@ -11786,7 +11786,7 @@
         <v>1338</v>
       </c>
     </row>
-    <row r="448" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="448" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A448" t="s">
         <v>95</v>
       </c>
@@ -11809,7 +11809,7 @@
         <v>1338</v>
       </c>
     </row>
-    <row r="449" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="449" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A449" t="s">
         <v>95</v>
       </c>
@@ -11832,7 +11832,7 @@
         <v>1338</v>
       </c>
     </row>
-    <row r="450" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="450" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A450" t="s">
         <v>95</v>
       </c>
@@ -11858,7 +11858,7 @@
         <v>1338</v>
       </c>
     </row>
-    <row r="451" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="451" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A451" t="s">
         <v>95</v>
       </c>
@@ -11881,7 +11881,7 @@
         <v>1338</v>
       </c>
     </row>
-    <row r="452" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="452" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A452" t="s">
         <v>95</v>
       </c>
@@ -11904,7 +11904,7 @@
         <v>1338</v>
       </c>
     </row>
-    <row r="453" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="453" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A453" t="s">
         <v>95</v>
       </c>
@@ -11927,7 +11927,7 @@
         <v>1338</v>
       </c>
     </row>
-    <row r="454" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="454" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A454" t="s">
         <v>95</v>
       </c>
@@ -11953,7 +11953,7 @@
         <v>1338</v>
       </c>
     </row>
-    <row r="455" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="455" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A455" t="s">
         <v>95</v>
       </c>
@@ -13869,7 +13869,7 @@
         <v>3293</v>
       </c>
     </row>
-    <row r="531" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="531" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A531" t="s">
         <v>116</v>
       </c>
@@ -13895,7 +13895,7 @@
         <v>2515</v>
       </c>
     </row>
-    <row r="532" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="532" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A532" t="s">
         <v>116</v>
       </c>
@@ -13921,7 +13921,7 @@
         <v>2515</v>
       </c>
     </row>
-    <row r="533" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="533" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A533" t="s">
         <v>116</v>
       </c>
@@ -13947,7 +13947,7 @@
         <v>2515</v>
       </c>
     </row>
-    <row r="534" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="534" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A534" t="s">
         <v>116</v>
       </c>
@@ -13973,7 +13973,7 @@
         <v>2515</v>
       </c>
     </row>
-    <row r="535" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="535" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A535" t="s">
         <v>116</v>
       </c>
@@ -13999,7 +13999,7 @@
         <v>2515</v>
       </c>
     </row>
-    <row r="536" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="536" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A536" t="s">
         <v>116</v>
       </c>
@@ -14025,7 +14025,7 @@
         <v>2515</v>
       </c>
     </row>
-    <row r="537" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="537" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A537" t="s">
         <v>116</v>
       </c>
@@ -14051,7 +14051,7 @@
         <v>2515</v>
       </c>
     </row>
-    <row r="538" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="538" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A538" t="s">
         <v>116</v>
       </c>
@@ -14077,7 +14077,7 @@
         <v>2515</v>
       </c>
     </row>
-    <row r="539" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="539" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A539" t="s">
         <v>116</v>
       </c>
@@ -14103,7 +14103,7 @@
         <v>2515</v>
       </c>
     </row>
-    <row r="540" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="540" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A540" t="s">
         <v>116</v>
       </c>
@@ -14884,10 +14884,18 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="D1:D569" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="0">
+  <autoFilter ref="A1:H569" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="3">
       <filters>
         <filter val="Italy"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="4">
+      <filters>
+        <filter val="Access to Adequate Assistance and Representation"/>
+        <filter val="Contacted an Advisor"/>
+        <filter val="National"/>
+        <filter val="Type of Advisor / Reason for No Contact"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -14896,26 +14904,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="46f3a809-46a3-44ee-a0f1-42a271529c86">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="69276225-f05c-44c5-92dc-c999460a4149" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006BF094976B1C6245BAB5BCECAC284645" ma:contentTypeVersion="17" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="de659102f67f900a4507bbf2a4959426">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="69276225-f05c-44c5-92dc-c999460a4149" xmlns:ns3="46f3a809-46a3-44ee-a0f1-42a271529c86" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9b8ee336b2a1d24b8ead4191187077de" ns2:_="" ns3:_="">
     <xsd:import namespace="69276225-f05c-44c5-92dc-c999460a4149"/>
@@ -15164,32 +15152,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B008726B-D02E-421E-93A7-4601A28BE471}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="69276225-f05c-44c5-92dc-c999460a4149"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="46f3a809-46a3-44ee-a0f1-42a271529c86"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{610EAA8D-4453-4809-85E4-2F8E1B9FB6D9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="46f3a809-46a3-44ee-a0f1-42a271529c86">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="69276225-f05c-44c5-92dc-c999460a4149" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A2D2E79F-2042-4968-909D-68BB0CA0DBF4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -15206,4 +15189,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{610EAA8D-4453-4809-85E4-2F8E1B9FB6D9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B008726B-D02E-421E-93A7-4601A28BE471}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="69276225-f05c-44c5-92dc-c999460a4149"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="46f3a809-46a3-44ee-a0f1-42a271529c86"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>